<commit_message>
Iterations 2 and 3
</commit_message>
<xml_diff>
--- a/Model.xlsx
+++ b/Model.xlsx
@@ -458,10 +458,10 @@
         <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>1.423370116707344</v>
+        <v>1.497142164392765</v>
       </c>
       <c r="E2" t="n">
-        <v>0.9589580027512145</v>
+        <v>1.058943747620302</v>
       </c>
     </row>
     <row r="3">
@@ -479,10 +479,10 @@
         <v>3</v>
       </c>
       <c r="D3" t="n">
-        <v>2.556852314434217</v>
+        <v>2.586322750169416</v>
       </c>
       <c r="E3" t="n">
-        <v>1.880731511478521</v>
+        <v>1.954383593348469</v>
       </c>
     </row>
     <row r="4">
@@ -500,10 +500,10 @@
         <v>6</v>
       </c>
       <c r="D4" t="n">
-        <v>3.82836256045553</v>
+        <v>3.877043778226711</v>
       </c>
       <c r="E4" t="n">
-        <v>3.063841689609428</v>
+        <v>3.150918239480372</v>
       </c>
     </row>
     <row r="5">
@@ -521,10 +521,10 @@
         <v>12</v>
       </c>
       <c r="D5" t="n">
-        <v>6.201078946604151</v>
+        <v>6.130910090836965</v>
       </c>
       <c r="E5" t="n">
-        <v>5.397666793147651</v>
+        <v>5.326871953296106</v>
       </c>
     </row>
     <row r="6">
@@ -542,10 +542,10 @@
         <v>24</v>
       </c>
       <c r="D6" t="n">
-        <v>9.807946506595533</v>
+        <v>8.445514176124318</v>
       </c>
       <c r="E6" t="n">
-        <v>8.6662982370676</v>
+        <v>7.355222876625018</v>
       </c>
     </row>
     <row r="7">
@@ -563,10 +563,10 @@
         <v>48</v>
       </c>
       <c r="D7" t="n">
-        <v>11.46148992696686</v>
+        <v>9.476547957699797</v>
       </c>
       <c r="E7" t="n">
-        <v>10.26593639618966</v>
+        <v>8.158333344391073</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Standardizing and horizon splitting
</commit_message>
<xml_diff>
--- a/Model.xlsx
+++ b/Model.xlsx
@@ -451,17 +451,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2025-01-01 to 2025-03-07</t>
+          <t>2024-01-01 to 2025-03-07</t>
         </is>
       </c>
       <c r="C2" t="n">
         <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>1.497142164392765</v>
+        <v>1.333784680835275</v>
       </c>
       <c r="E2" t="n">
-        <v>1.058943747620302</v>
+        <v>0.9930298346466162</v>
       </c>
     </row>
     <row r="3">
@@ -472,17 +472,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2025-01-01 to 2025-03-07</t>
+          <t>2024-01-01 to 2025-03-07</t>
         </is>
       </c>
       <c r="C3" t="n">
         <v>3</v>
       </c>
       <c r="D3" t="n">
-        <v>2.586322750169416</v>
+        <v>2.44476863628705</v>
       </c>
       <c r="E3" t="n">
-        <v>1.954383593348469</v>
+        <v>1.888550762178128</v>
       </c>
     </row>
     <row r="4">
@@ -493,17 +493,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2025-01-01 to 2025-03-07</t>
+          <t>2024-01-01 to 2025-03-07</t>
         </is>
       </c>
       <c r="C4" t="n">
         <v>6</v>
       </c>
       <c r="D4" t="n">
-        <v>3.877043778226711</v>
+        <v>3.704616831277799</v>
       </c>
       <c r="E4" t="n">
-        <v>3.150918239480372</v>
+        <v>2.89599108398655</v>
       </c>
     </row>
     <row r="5">
@@ -514,17 +514,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2025-01-01 to 2025-03-07</t>
+          <t>2024-01-01 to 2025-03-07</t>
         </is>
       </c>
       <c r="C5" t="n">
         <v>12</v>
       </c>
       <c r="D5" t="n">
-        <v>6.130910090836965</v>
+        <v>4.991566614690754</v>
       </c>
       <c r="E5" t="n">
-        <v>5.326871953296106</v>
+        <v>3.919764193792211</v>
       </c>
     </row>
     <row r="6">
@@ -535,17 +535,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2025-01-01 to 2025-03-07</t>
+          <t>2024-01-01 to 2025-03-07</t>
         </is>
       </c>
       <c r="C6" t="n">
         <v>24</v>
       </c>
       <c r="D6" t="n">
-        <v>8.445514176124318</v>
+        <v>5.942686113030913</v>
       </c>
       <c r="E6" t="n">
-        <v>7.355222876625018</v>
+        <v>4.769132139989177</v>
       </c>
     </row>
     <row r="7">
@@ -556,17 +556,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2025-01-01 to 2025-03-07</t>
+          <t>2024-01-01 to 2025-03-07</t>
         </is>
       </c>
       <c r="C7" t="n">
         <v>48</v>
       </c>
       <c r="D7" t="n">
-        <v>9.476547957699797</v>
+        <v>6.539251016446201</v>
       </c>
       <c r="E7" t="n">
-        <v>8.158333344391073</v>
+        <v>5.338850861819732</v>
       </c>
     </row>
   </sheetData>

</xml_diff>